<commit_message>
aanpassing juni 1 les
aanpassing om in juni 1 les te houden die langer duurt
</commit_message>
<xml_diff>
--- a/flyers/Mechelen_2025-26.xlsx
+++ b/flyers/Mechelen_2025-26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joachim/Sites/EddyPresent18/flyers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75195B53-C40D-854A-B908-0D9F0934AD36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37B0B123-A13D-2A4F-8242-4E2BC1C44C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="30240" windowHeight="17840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16320" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="31">
   <si>
     <t>Dag</t>
   </si>
@@ -130,12 +130,15 @@
   <si>
     <t>Eddy of Marc</t>
   </si>
+  <si>
+    <t>1 Les</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -166,6 +169,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -352,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -510,9 +520,43 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium7"/>
@@ -3879,12 +3923,12 @@
       </c>
       <c r="I107" s="22"/>
       <c r="J107" s="9"/>
-      <c r="K107" s="23"/>
-      <c r="L107" s="21"/>
-      <c r="M107" s="21" t="s">
+      <c r="K107" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="N107" s="22"/>
+      <c r="L107" s="63"/>
+      <c r="M107" s="63"/>
+      <c r="N107" s="65"/>
     </row>
     <row r="108" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="28" t="s">
@@ -3913,12 +3957,10 @@
         <v>0</v>
       </c>
       <c r="L108" s="30"/>
-      <c r="M108" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="N108" s="26" t="s">
-        <v>9</v>
-      </c>
+      <c r="M108" s="62" t="s">
+        <v>30</v>
+      </c>
+      <c r="N108" s="57"/>
     </row>
     <row r="109" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="3" t="s">
@@ -4037,12 +4079,10 @@
       <c r="L112" s="10">
         <v>4</v>
       </c>
-      <c r="M112" s="36" t="s">
-        <v>10</v>
-      </c>
-      <c r="N112" s="34" t="s">
-        <v>10</v>
-      </c>
+      <c r="M112" s="58" t="s">
+        <v>10</v>
+      </c>
+      <c r="N112" s="59"/>
     </row>
     <row r="113" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="3" t="s">
@@ -4249,12 +4289,10 @@
       <c r="L119" s="10">
         <v>11</v>
       </c>
-      <c r="M119" s="39" t="s">
-        <v>11</v>
-      </c>
-      <c r="N119" s="38" t="s">
-        <v>11</v>
-      </c>
+      <c r="M119" s="60" t="s">
+        <v>11</v>
+      </c>
+      <c r="N119" s="61"/>
     </row>
     <row r="120" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="3" t="s">
@@ -4461,12 +4499,10 @@
       <c r="L126" s="10">
         <v>18</v>
       </c>
-      <c r="M126" s="36" t="s">
-        <v>10</v>
-      </c>
-      <c r="N126" s="34" t="s">
-        <v>10</v>
-      </c>
+      <c r="M126" s="58" t="s">
+        <v>10</v>
+      </c>
+      <c r="N126" s="59"/>
       <c r="O126" s="8"/>
     </row>
     <row r="127" spans="1:15" ht="12" customHeight="1" x14ac:dyDescent="0.2">
@@ -4918,6 +4954,13 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="M108:N108"/>
+    <mergeCell ref="M112:N112"/>
+    <mergeCell ref="M119:N119"/>
+    <mergeCell ref="M126:N126"/>
+    <mergeCell ref="K107:N107"/>
+  </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.5" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="3"/>

</xml_diff>